<commit_message>
feat(engine): redefine borderline as the in-range cusp
Borderline now means a value is still INSIDE the reference range but
within the outer ~15% margin of a boundary — i.e. on the cusp of
leaving the in-range zone (an early warning), rather than a band just
outside the range. Anything outside the range is out-of-range/critical.

- buildLabRanges.js: Borderline Low/High become the inner comfortable-core
  thresholds (CUSP_FRACTION of the in-range span), directional so the low
  cusp is skipped on nominal-0 floors and the high cusp on open-ended limits.
- classify.js: classifyExplicit + legacy classify updated to the cusp rule.
- Lab_Ranges.xlsx regenerated (159 rows, 0 geometry violations).
- Engine prompt §1B tier table updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Lab_Ranges.xlsx
+++ b/Data/Lab_Ranges.xlsx
@@ -467,10 +467,10 @@
         <v>11</v>
       </c>
       <c r="G2">
-        <v>4.05</v>
+        <v>5.475</v>
       </c>
       <c r="H2">
-        <v>12.1</v>
+        <v>10.025</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -502,10 +502,10 @@
         <v>5.9</v>
       </c>
       <c r="G3">
-        <v>4.05</v>
+        <v>4.71</v>
       </c>
       <c r="H3">
-        <v>6.49</v>
+        <v>5.69</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -531,10 +531,10 @@
         <v>5.2</v>
       </c>
       <c r="G4">
-        <v>3.6</v>
+        <v>4.18</v>
       </c>
       <c r="H4">
-        <v>5.72</v>
+        <v>5.02</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -560,10 +560,10 @@
         <v>17.5</v>
       </c>
       <c r="G5">
-        <v>12.15</v>
+        <v>14.1</v>
       </c>
       <c r="H5">
-        <v>19.25</v>
+        <v>16.9</v>
       </c>
       <c r="I5">
         <v>7</v>
@@ -595,10 +595,10 @@
         <v>15.5</v>
       </c>
       <c r="G6">
-        <v>10.8</v>
+        <v>12.525</v>
       </c>
       <c r="H6">
-        <v>17.05</v>
+        <v>14.975</v>
       </c>
       <c r="I6">
         <v>7</v>
@@ -630,10 +630,10 @@
         <v>53</v>
       </c>
       <c r="G7">
-        <v>36.9</v>
+        <v>42.8</v>
       </c>
       <c r="H7">
-        <v>58.3</v>
+        <v>51.2</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -659,10 +659,10 @@
         <v>46</v>
       </c>
       <c r="G8">
-        <v>32.4</v>
+        <v>37.5</v>
       </c>
       <c r="H8">
-        <v>50.6</v>
+        <v>44.5</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -688,10 +688,10 @@
         <v>100</v>
       </c>
       <c r="G9">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="H9">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -717,10 +717,10 @@
         <v>33</v>
       </c>
       <c r="G10">
-        <v>24.3</v>
+        <v>27.9</v>
       </c>
       <c r="H10">
-        <v>36.3</v>
+        <v>32.1</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -746,10 +746,10 @@
         <v>36</v>
       </c>
       <c r="G11">
-        <v>28.8</v>
+        <v>32.6</v>
       </c>
       <c r="H11">
-        <v>39.6</v>
+        <v>35.4</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -775,10 +775,10 @@
         <v>14.5</v>
       </c>
       <c r="G12">
-        <v>10.35</v>
+        <v>11.95</v>
       </c>
       <c r="H12">
-        <v>15.95</v>
+        <v>14.05</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -804,10 +804,10 @@
         <v>400</v>
       </c>
       <c r="G13">
-        <v>135</v>
+        <v>187.5</v>
       </c>
       <c r="H13">
-        <v>440</v>
+        <v>362.5</v>
       </c>
       <c r="I13">
         <v>20</v>
@@ -839,10 +839,10 @@
         <v>70</v>
       </c>
       <c r="G14">
-        <v>36</v>
+        <v>44.5</v>
       </c>
       <c r="H14">
-        <v>77</v>
+        <v>65.5</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -868,10 +868,10 @@
         <v>40</v>
       </c>
       <c r="G15">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H15">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -897,10 +897,10 @@
         <v>10</v>
       </c>
       <c r="G16">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="H16">
-        <v>11</v>
+        <v>8.8</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -926,10 +926,10 @@
         <v>4</v>
       </c>
       <c r="G17">
-        <v>0.9</v>
+        <v>1.45</v>
       </c>
       <c r="H17">
-        <v>4.4</v>
+        <v>3.55</v>
       </c>
       <c r="K17" t="str">
         <v/>
@@ -955,7 +955,7 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>1.1</v>
+        <v>0.85</v>
       </c>
       <c r="K18" t="str">
         <v/>
@@ -981,10 +981,10 @@
         <v>99</v>
       </c>
       <c r="G19">
-        <v>60</v>
+        <v>74.35</v>
       </c>
       <c r="H19">
-        <v>125</v>
+        <v>94.65</v>
       </c>
       <c r="I19">
         <v>50</v>
@@ -1016,10 +1016,10 @@
         <v>5.6</v>
       </c>
       <c r="G20">
-        <v>3.6</v>
+        <v>4.24</v>
       </c>
       <c r="H20">
-        <v>6.4</v>
+        <v>5.36</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -1045,7 +1045,7 @@
         <v>199</v>
       </c>
       <c r="H21">
-        <v>239</v>
+        <v>169.15</v>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -1071,7 +1071,7 @@
         <v>99</v>
       </c>
       <c r="H22">
-        <v>159</v>
+        <v>84.15</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -1097,7 +1097,7 @@
         <v>999</v>
       </c>
       <c r="G23">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="K23" t="str">
         <v>Lower bound is the risk threshold; higher is protective.</v>
@@ -1123,7 +1123,7 @@
         <v>999</v>
       </c>
       <c r="G24">
-        <v>45</v>
+        <v>57.5</v>
       </c>
       <c r="K24" t="str">
         <v>Lower bound is the risk threshold; higher is protective.</v>
@@ -1149,7 +1149,7 @@
         <v>149</v>
       </c>
       <c r="H25">
-        <v>199</v>
+        <v>126.65</v>
       </c>
       <c r="J25">
         <v>1000</v>
@@ -1178,7 +1178,7 @@
         <v>1</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>0.85</v>
       </c>
       <c r="K26" t="str">
         <v>Cardiac risk: &lt;1 low, 1-3 average, &gt;3 high.</v>
@@ -1204,10 +1204,10 @@
         <v>56</v>
       </c>
       <c r="G27">
-        <v>6.3</v>
+        <v>14.35</v>
       </c>
       <c r="H27">
-        <v>61.6</v>
+        <v>48.65</v>
       </c>
       <c r="J27">
         <v>500</v>
@@ -1236,10 +1236,10 @@
         <v>40</v>
       </c>
       <c r="G28">
-        <v>9</v>
+        <v>14.5</v>
       </c>
       <c r="H28">
-        <v>44</v>
+        <v>35.5</v>
       </c>
       <c r="J28">
         <v>500</v>
@@ -1268,10 +1268,10 @@
         <v>147</v>
       </c>
       <c r="G29">
-        <v>39.6</v>
+        <v>59.45</v>
       </c>
       <c r="H29">
-        <v>161.7</v>
+        <v>131.55</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -1297,10 +1297,10 @@
         <v>1.2</v>
       </c>
       <c r="G30">
-        <v>0.09</v>
+        <v>0.265</v>
       </c>
       <c r="H30">
-        <v>1.32</v>
+        <v>1.035</v>
       </c>
       <c r="J30">
         <v>15</v>
@@ -1329,7 +1329,7 @@
         <v>0.3</v>
       </c>
       <c r="H31">
-        <v>0.33</v>
+        <v>0.255</v>
       </c>
       <c r="K31" t="str">
         <v/>
@@ -1355,10 +1355,10 @@
         <v>0.9</v>
       </c>
       <c r="G32">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="H32">
-        <v>0.99</v>
+        <v>0.78</v>
       </c>
       <c r="K32" t="str">
         <v/>
@@ -1384,10 +1384,10 @@
         <v>5</v>
       </c>
       <c r="G33">
-        <v>3.15</v>
+        <v>3.725</v>
       </c>
       <c r="H33">
-        <v>5.5</v>
+        <v>4.775</v>
       </c>
       <c r="K33" t="str">
         <v/>
@@ -1413,10 +1413,10 @@
         <v>8.5</v>
       </c>
       <c r="G34">
-        <v>5.4</v>
+        <v>6.375</v>
       </c>
       <c r="H34">
-        <v>9.35</v>
+        <v>8.125</v>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -1442,10 +1442,10 @@
         <v>1.35</v>
       </c>
       <c r="G35">
-        <v>0.666</v>
+        <v>0.832</v>
       </c>
       <c r="H35">
-        <v>1.485</v>
+        <v>1.259</v>
       </c>
       <c r="J35">
         <v>10</v>
@@ -1474,10 +1474,10 @@
         <v>1.04</v>
       </c>
       <c r="G36">
-        <v>0.531</v>
+        <v>0.658</v>
       </c>
       <c r="H36">
-        <v>1.144</v>
+        <v>0.973</v>
       </c>
       <c r="J36">
         <v>10</v>
@@ -1506,10 +1506,10 @@
         <v>20</v>
       </c>
       <c r="G37">
-        <v>6.3</v>
+        <v>8.95</v>
       </c>
       <c r="H37">
-        <v>22</v>
+        <v>18.05</v>
       </c>
       <c r="J37">
         <v>100</v>
@@ -1573,10 +1573,10 @@
         <v>10.5</v>
       </c>
       <c r="G39">
-        <v>7.65</v>
+        <v>8.8</v>
       </c>
       <c r="H39">
-        <v>11.55</v>
+        <v>10.2</v>
       </c>
       <c r="I39">
         <v>6</v>
@@ -1608,10 +1608,10 @@
         <v>2.2</v>
       </c>
       <c r="G40">
-        <v>1.53</v>
+        <v>1.775</v>
       </c>
       <c r="H40">
-        <v>2.42</v>
+        <v>2.125</v>
       </c>
       <c r="I40">
         <v>1</v>
@@ -1643,10 +1643,10 @@
         <v>5.1</v>
       </c>
       <c r="G41">
-        <v>3.15</v>
+        <v>3.74</v>
       </c>
       <c r="H41">
-        <v>5.61</v>
+        <v>4.86</v>
       </c>
       <c r="I41">
         <v>2.5</v>
@@ -1678,10 +1678,10 @@
         <v>145</v>
       </c>
       <c r="G42">
-        <v>122.4</v>
+        <v>137.35</v>
       </c>
       <c r="H42">
-        <v>159.5</v>
+        <v>143.65</v>
       </c>
       <c r="I42">
         <v>120</v>
@@ -1713,10 +1713,10 @@
         <v>107</v>
       </c>
       <c r="G43">
-        <v>88.2</v>
+        <v>99.35</v>
       </c>
       <c r="H43">
-        <v>117.7</v>
+        <v>105.65</v>
       </c>
       <c r="I43">
         <v>80</v>
@@ -1748,10 +1748,10 @@
         <v>4.5</v>
       </c>
       <c r="G44">
-        <v>2.25</v>
+        <v>2.8</v>
       </c>
       <c r="H44">
-        <v>4.95</v>
+        <v>4.2</v>
       </c>
       <c r="K44" t="str">
         <v/>
@@ -1777,10 +1777,10 @@
         <v>29</v>
       </c>
       <c r="G45">
-        <v>19.8</v>
+        <v>23.05</v>
       </c>
       <c r="H45">
-        <v>31.9</v>
+        <v>27.95</v>
       </c>
       <c r="I45">
         <v>10</v>
@@ -1812,10 +1812,10 @@
         <v>4.5</v>
       </c>
       <c r="G46">
-        <v>0.1</v>
+        <v>1.057</v>
       </c>
       <c r="H46">
-        <v>10</v>
+        <v>3.893</v>
       </c>
       <c r="I46">
         <v>0.01</v>
@@ -1847,10 +1847,10 @@
         <v>7</v>
       </c>
       <c r="G47">
-        <v>3.06</v>
+        <v>3.94</v>
       </c>
       <c r="H47">
-        <v>8</v>
+        <v>6.46</v>
       </c>
       <c r="K47" t="str">
         <v/>
@@ -1876,10 +1876,10 @@
         <v>6</v>
       </c>
       <c r="G48">
-        <v>2.16</v>
+        <v>2.94</v>
       </c>
       <c r="H48">
-        <v>8</v>
+        <v>5.46</v>
       </c>
       <c r="K48" t="str">
         <v/>
@@ -1905,9 +1905,12 @@
         <v>100</v>
       </c>
       <c r="G49">
-        <v>20</v>
+        <v>40.5</v>
       </c>
       <c r="H49">
+        <v>89.5</v>
+      </c>
+      <c r="J49">
         <v>150</v>
       </c>
       <c r="K49" t="str">
@@ -1934,10 +1937,10 @@
         <v>400</v>
       </c>
       <c r="G50">
-        <v>27</v>
+        <v>85.5</v>
       </c>
       <c r="H50">
-        <v>440</v>
+        <v>344.5</v>
       </c>
       <c r="K50" t="str">
         <v/>
@@ -1963,10 +1966,10 @@
         <v>150</v>
       </c>
       <c r="G51">
-        <v>11.7</v>
+        <v>33.55</v>
       </c>
       <c r="H51">
-        <v>165</v>
+        <v>129.45</v>
       </c>
       <c r="K51" t="str">
         <v/>
@@ -1992,7 +1995,7 @@
         <v>90</v>
       </c>
       <c r="H52">
-        <v>99</v>
+        <v>76.5</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -2018,7 +2021,7 @@
         <v>30</v>
       </c>
       <c r="H53">
-        <v>33</v>
+        <v>25.5</v>
       </c>
       <c r="K53" t="str">
         <v>~&lt;75 nmol/L equivalent.</v>
@@ -2044,7 +2047,7 @@
         <v>99</v>
       </c>
       <c r="H54">
-        <v>159</v>
+        <v>84.15</v>
       </c>
       <c r="K54" t="str">
         <v/>
@@ -2070,7 +2073,7 @@
         <v>35</v>
       </c>
       <c r="H55">
-        <v>38.5</v>
+        <v>29.75</v>
       </c>
       <c r="K55" t="str">
         <v>Optimal &lt;20; borderline 20-40; high &gt;40 (web research).</v>
@@ -2119,7 +2122,7 @@
         <v>999</v>
       </c>
       <c r="G57">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="K57" t="str">
         <v/>
@@ -2145,7 +2148,7 @@
         <v>999</v>
       </c>
       <c r="G58">
-        <v>45</v>
+        <v>57.5</v>
       </c>
       <c r="K58" t="str">
         <v/>
@@ -2171,10 +2174,10 @@
         <v>30</v>
       </c>
       <c r="G59">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H59">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="K59" t="str">
         <v>NMR subfraction; higher = more protective. Range approximate/assay-dependent.</v>
@@ -2200,10 +2203,10 @@
         <v>40</v>
       </c>
       <c r="G60">
-        <v>4.5</v>
+        <v>10.25</v>
       </c>
       <c r="H60">
-        <v>44</v>
+        <v>34.75</v>
       </c>
       <c r="K60" t="str">
         <v/>
@@ -2229,7 +2232,7 @@
         <v>15</v>
       </c>
       <c r="H61">
-        <v>20</v>
+        <v>12.75</v>
       </c>
       <c r="K61" t="str">
         <v>Optimal &lt;10.</v>
@@ -2255,7 +2258,7 @@
         <v>125</v>
       </c>
       <c r="H62">
-        <v>137.5</v>
+        <v>106.25</v>
       </c>
       <c r="K62" t="str">
         <v>Outpatient cutoff &lt;125 (&lt;75 yr); age-adjusted acute HF cutoffs higher.</v>
@@ -2281,7 +2284,7 @@
         <v>3</v>
       </c>
       <c r="H63">
-        <v>3.3</v>
+        <v>2.55</v>
       </c>
       <c r="K63" t="str">
         <v>Optimal &lt;2.0; insulin-resistance surrogate.</v>
@@ -2307,10 +2310,10 @@
         <v>916</v>
       </c>
       <c r="G64">
-        <v>237.6</v>
+        <v>361.8</v>
       </c>
       <c r="H64">
-        <v>1007.6</v>
+        <v>818.2</v>
       </c>
       <c r="K64" t="str">
         <v/>
@@ -2336,10 +2339,10 @@
         <v>70</v>
       </c>
       <c r="G65">
-        <v>13.5</v>
+        <v>23.25</v>
       </c>
       <c r="H65">
-        <v>77</v>
+        <v>61.75</v>
       </c>
       <c r="K65" t="str">
         <v/>
@@ -2365,10 +2368,10 @@
         <v>26.5</v>
       </c>
       <c r="G66">
-        <v>8.37</v>
+        <v>11.88</v>
       </c>
       <c r="H66">
-        <v>29.15</v>
+        <v>23.92</v>
       </c>
       <c r="K66" t="str">
         <v/>
@@ -2394,10 +2397,10 @@
         <v>6.8</v>
       </c>
       <c r="G67">
-        <v>0.54</v>
+        <v>1.53</v>
       </c>
       <c r="H67">
-        <v>7.48</v>
+        <v>5.87</v>
       </c>
       <c r="K67" t="str">
         <v/>
@@ -2423,10 +2426,10 @@
         <v>42.6</v>
       </c>
       <c r="G68">
-        <v>6.84</v>
+        <v>12.85</v>
       </c>
       <c r="H68">
-        <v>46.86</v>
+        <v>37.35</v>
       </c>
       <c r="K68" t="str">
         <v>Female varies by menstrual phase.</v>
@@ -2452,10 +2455,10 @@
         <v>166</v>
       </c>
       <c r="G69">
-        <v>11.25</v>
+        <v>35.525</v>
       </c>
       <c r="H69">
-        <v>182.6</v>
+        <v>142.975</v>
       </c>
       <c r="K69" t="str">
         <v>Female varies by menstrual phase.</v>
@@ -2481,10 +2484,10 @@
         <v>12.4</v>
       </c>
       <c r="G70">
-        <v>1.35</v>
+        <v>3.135</v>
       </c>
       <c r="H70">
-        <v>13.64</v>
+        <v>10.765</v>
       </c>
       <c r="K70" t="str">
         <v/>
@@ -2510,10 +2513,10 @@
         <v>20</v>
       </c>
       <c r="G71">
-        <v>2.7</v>
+        <v>5.55</v>
       </c>
       <c r="H71">
-        <v>22</v>
+        <v>17.45</v>
       </c>
       <c r="K71" t="str">
         <v/>
@@ -2539,10 +2542,10 @@
         <v>8.6</v>
       </c>
       <c r="G72">
-        <v>1.53</v>
+        <v>2.735</v>
       </c>
       <c r="H72">
-        <v>9.46</v>
+        <v>7.565</v>
       </c>
       <c r="K72" t="str">
         <v/>
@@ -2568,10 +2571,10 @@
         <v>18</v>
       </c>
       <c r="G73">
-        <v>0.9</v>
+        <v>3.55</v>
       </c>
       <c r="H73">
-        <v>19.8</v>
+        <v>15.45</v>
       </c>
       <c r="K73" t="str">
         <v/>
@@ -2597,10 +2600,10 @@
         <v>18</v>
       </c>
       <c r="G74">
-        <v>1.8</v>
+        <v>4.4</v>
       </c>
       <c r="H74">
-        <v>19.8</v>
+        <v>15.6</v>
       </c>
       <c r="K74" t="str">
         <v/>
@@ -2626,10 +2629,10 @@
         <v>29.2</v>
       </c>
       <c r="G75">
-        <v>2.52</v>
+        <v>6.76</v>
       </c>
       <c r="H75">
-        <v>32.12</v>
+        <v>25.24</v>
       </c>
       <c r="K75" t="str">
         <v/>
@@ -2655,7 +2658,7 @@
         <v>4</v>
       </c>
       <c r="H76">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="K76" t="str">
         <v>Male; age-adjusted upper limits exist.</v>
@@ -2681,10 +2684,10 @@
         <v>100</v>
       </c>
       <c r="G77">
-        <v>22.5</v>
+        <v>36.25</v>
       </c>
       <c r="H77">
-        <v>110</v>
+        <v>88.75</v>
       </c>
       <c r="K77" t="str">
         <v>% free of total PSA; &gt;25% favorable, &lt;10% higher risk.</v>
@@ -2710,10 +2713,10 @@
         <v>57</v>
       </c>
       <c r="G78">
-        <v>9</v>
+        <v>17.05</v>
       </c>
       <c r="H78">
-        <v>62.7</v>
+        <v>49.95</v>
       </c>
       <c r="K78" t="str">
         <v/>
@@ -2739,10 +2742,10 @@
         <v>144</v>
       </c>
       <c r="G79">
-        <v>16.2</v>
+        <v>36.9</v>
       </c>
       <c r="H79">
-        <v>158.4</v>
+        <v>125.1</v>
       </c>
       <c r="K79" t="str">
         <v/>
@@ -2768,10 +2771,10 @@
         <v>42.6</v>
       </c>
       <c r="G80">
-        <v>6.84</v>
+        <v>12.85</v>
       </c>
       <c r="H80">
-        <v>46.86</v>
+        <v>37.35</v>
       </c>
       <c r="K80" t="str">
         <v>Female varies by menstrual phase.</v>
@@ -2797,10 +2800,10 @@
         <v>166</v>
       </c>
       <c r="G81">
-        <v>11.25</v>
+        <v>35.525</v>
       </c>
       <c r="H81">
-        <v>182.6</v>
+        <v>142.975</v>
       </c>
       <c r="K81" t="str">
         <v>Female varies by menstrual phase.</v>
@@ -2826,10 +2829,10 @@
         <v>25</v>
       </c>
       <c r="G82">
-        <v>0.09</v>
+        <v>3.835</v>
       </c>
       <c r="H82">
-        <v>27.5</v>
+        <v>21.265</v>
       </c>
       <c r="K82" t="str">
         <v>Female; follicular &lt;1.5, luteal 2-25 (phase-dependent).</v>
@@ -2855,10 +2858,10 @@
         <v>12.4</v>
       </c>
       <c r="G83">
-        <v>1.35</v>
+        <v>3.135</v>
       </c>
       <c r="H83">
-        <v>13.64</v>
+        <v>10.765</v>
       </c>
       <c r="K83" t="str">
         <v/>
@@ -2884,10 +2887,10 @@
         <v>20</v>
       </c>
       <c r="G84">
-        <v>2.7</v>
+        <v>5.55</v>
       </c>
       <c r="H84">
-        <v>22</v>
+        <v>17.45</v>
       </c>
       <c r="K84" t="str">
         <v/>
@@ -2913,10 +2916,10 @@
         <v>8.6</v>
       </c>
       <c r="G85">
-        <v>1.53</v>
+        <v>2.735</v>
       </c>
       <c r="H85">
-        <v>9.46</v>
+        <v>7.565</v>
       </c>
       <c r="K85" t="str">
         <v/>
@@ -2942,10 +2945,10 @@
         <v>18</v>
       </c>
       <c r="G86">
-        <v>0.9</v>
+        <v>3.55</v>
       </c>
       <c r="H86">
-        <v>19.8</v>
+        <v>15.45</v>
       </c>
       <c r="K86" t="str">
         <v/>
@@ -2971,10 +2974,10 @@
         <v>18</v>
       </c>
       <c r="G87">
-        <v>1.8</v>
+        <v>4.4</v>
       </c>
       <c r="H87">
-        <v>19.8</v>
+        <v>15.6</v>
       </c>
       <c r="K87" t="str">
         <v/>
@@ -3000,10 +3003,10 @@
         <v>29.2</v>
       </c>
       <c r="G88">
-        <v>2.52</v>
+        <v>6.76</v>
       </c>
       <c r="H88">
-        <v>32.12</v>
+        <v>25.24</v>
       </c>
       <c r="K88" t="str">
         <v/>
@@ -3029,10 +3032,10 @@
         <v>57</v>
       </c>
       <c r="G89">
-        <v>9</v>
+        <v>17.05</v>
       </c>
       <c r="H89">
-        <v>62.7</v>
+        <v>49.95</v>
       </c>
       <c r="K89" t="str">
         <v/>
@@ -3058,10 +3061,10 @@
         <v>144</v>
       </c>
       <c r="G90">
-        <v>16.2</v>
+        <v>36.9</v>
       </c>
       <c r="H90">
-        <v>158.4</v>
+        <v>125.1</v>
       </c>
       <c r="K90" t="str">
         <v/>
@@ -3087,10 +3090,10 @@
         <v>510</v>
       </c>
       <c r="G91">
-        <v>99</v>
+        <v>170</v>
       </c>
       <c r="H91">
-        <v>561</v>
+        <v>450</v>
       </c>
       <c r="K91" t="str">
         <v>Declines ~2%/yr after age 25.</v>
@@ -3116,10 +3119,10 @@
         <v>320</v>
       </c>
       <c r="G92">
-        <v>40.5</v>
+        <v>86.25</v>
       </c>
       <c r="H92">
-        <v>352</v>
+        <v>278.75</v>
       </c>
       <c r="K92" t="str">
         <v>Declines ~2%/yr after age 25.</v>
@@ -3145,10 +3148,10 @@
         <v>916</v>
       </c>
       <c r="G93">
-        <v>237.6</v>
+        <v>361.8</v>
       </c>
       <c r="H93">
-        <v>1007.6</v>
+        <v>818.2</v>
       </c>
       <c r="K93" t="str">
         <v/>
@@ -3174,10 +3177,10 @@
         <v>70</v>
       </c>
       <c r="G94">
-        <v>13.5</v>
+        <v>23.25</v>
       </c>
       <c r="H94">
-        <v>77</v>
+        <v>61.75</v>
       </c>
       <c r="K94" t="str">
         <v/>
@@ -3203,10 +3206,10 @@
         <v>3.5</v>
       </c>
       <c r="G95">
-        <v>0.9</v>
+        <v>1.375</v>
       </c>
       <c r="H95">
-        <v>3.85</v>
+        <v>3.125</v>
       </c>
       <c r="K95" t="str">
         <v>Female; age-dependent, declines with age (&lt;1.0 = low reserve).</v>
@@ -3232,10 +3235,10 @@
         <v>19.4</v>
       </c>
       <c r="G96">
-        <v>5.58</v>
+        <v>8.18</v>
       </c>
       <c r="H96">
-        <v>21.34</v>
+        <v>17.42</v>
       </c>
       <c r="K96" t="str">
         <v>AM sample (7-9am).</v>
@@ -3261,10 +3264,10 @@
         <v>4.5</v>
       </c>
       <c r="G97">
-        <v>0.1</v>
+        <v>1.057</v>
       </c>
       <c r="H97">
-        <v>10</v>
+        <v>3.893</v>
       </c>
       <c r="I97">
         <v>0.01</v>
@@ -3296,10 +3299,10 @@
         <v>4.4</v>
       </c>
       <c r="G98">
-        <v>1.8</v>
+        <v>2.36</v>
       </c>
       <c r="H98">
-        <v>4.84</v>
+        <v>4.04</v>
       </c>
       <c r="K98" t="str">
         <v/>
@@ -3325,10 +3328,10 @@
         <v>1.77</v>
       </c>
       <c r="G99">
-        <v>0.738</v>
+        <v>0.962</v>
       </c>
       <c r="H99">
-        <v>1.947</v>
+        <v>1.628</v>
       </c>
       <c r="K99" t="str">
         <v/>
@@ -3354,7 +3357,7 @@
         <v>34</v>
       </c>
       <c r="H100">
-        <v>37.4</v>
+        <v>28.9</v>
       </c>
       <c r="K100" t="str">
         <v/>
@@ -3380,7 +3383,7 @@
         <v>4</v>
       </c>
       <c r="H101">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="K101" t="str">
         <v>Assay-dependent (some report &lt;115).</v>
@@ -3406,10 +3409,10 @@
         <v>900</v>
       </c>
       <c r="G102">
-        <v>180</v>
+        <v>305</v>
       </c>
       <c r="H102">
-        <v>990</v>
+        <v>795</v>
       </c>
       <c r="K102" t="str">
         <v>Optimal &gt;500.</v>
@@ -3435,10 +3438,10 @@
         <v>17</v>
       </c>
       <c r="G103">
-        <v>2.7</v>
+        <v>5.1</v>
       </c>
       <c r="H103">
-        <v>18.7</v>
+        <v>14.9</v>
       </c>
       <c r="K103" t="str">
         <v/>
@@ -3464,10 +3467,10 @@
         <v>50</v>
       </c>
       <c r="G104">
-        <v>4.5</v>
+        <v>11.75</v>
       </c>
       <c r="H104">
-        <v>55</v>
+        <v>43.25</v>
       </c>
       <c r="K104" t="str">
         <v>As pyridoxal-5-phosphate (P5P).</v>
@@ -3493,10 +3496,10 @@
         <v>120</v>
       </c>
       <c r="G105">
-        <v>63</v>
+        <v>77.5</v>
       </c>
       <c r="H105">
-        <v>132</v>
+        <v>112.5</v>
       </c>
       <c r="K105" t="str">
         <v/>
@@ -3522,10 +3525,10 @@
         <v>155</v>
       </c>
       <c r="G106">
-        <v>72</v>
+        <v>91.25</v>
       </c>
       <c r="H106">
-        <v>170.5</v>
+        <v>143.75</v>
       </c>
       <c r="K106" t="str">
         <v/>
@@ -3551,10 +3554,10 @@
         <v>150</v>
       </c>
       <c r="G107">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="H107">
-        <v>165</v>
+        <v>138</v>
       </c>
       <c r="K107" t="str">
         <v/>
@@ -3580,10 +3583,10 @@
         <v>170</v>
       </c>
       <c r="G108">
-        <v>54</v>
+        <v>76.5</v>
       </c>
       <c r="H108">
-        <v>187</v>
+        <v>153.5</v>
       </c>
       <c r="K108" t="str">
         <v/>
@@ -3609,10 +3612,10 @@
         <v>370</v>
       </c>
       <c r="G109">
-        <v>225</v>
+        <v>268</v>
       </c>
       <c r="H109">
-        <v>407</v>
+        <v>352</v>
       </c>
       <c r="K109" t="str">
         <v/>
@@ -3638,10 +3641,10 @@
         <v>50</v>
       </c>
       <c r="G110">
-        <v>13.5</v>
+        <v>20.25</v>
       </c>
       <c r="H110">
-        <v>55</v>
+        <v>44.75</v>
       </c>
       <c r="K110" t="str">
         <v/>
@@ -3667,10 +3670,10 @@
         <v>12</v>
       </c>
       <c r="G111">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
       <c r="H111">
-        <v>13.2</v>
+        <v>11.4</v>
       </c>
       <c r="K111" t="str">
         <v>Target &gt;=8% (higher = lower CV risk); &lt;4% high risk.</v>
@@ -3696,10 +3699,10 @@
         <v>60</v>
       </c>
       <c r="G112">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H112">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="K112" t="str">
         <v/>
@@ -3725,10 +3728,10 @@
         <v>17</v>
       </c>
       <c r="G113">
-        <v>4.95</v>
+        <v>7.225</v>
       </c>
       <c r="H113">
-        <v>18.7</v>
+        <v>15.275</v>
       </c>
       <c r="K113" t="str">
         <v>Alpha-tocopherol.</v>
@@ -3754,10 +3757,10 @@
         <v>1.01</v>
       </c>
       <c r="G114">
-        <v>0.153</v>
+        <v>0.296</v>
       </c>
       <c r="H114">
-        <v>1.111</v>
+        <v>0.884</v>
       </c>
       <c r="K114" t="str">
         <v>MK-7; highly assay-dependent (web research).</v>
@@ -3783,10 +3786,10 @@
         <v>19.4</v>
       </c>
       <c r="G115">
-        <v>5.58</v>
+        <v>8.18</v>
       </c>
       <c r="H115">
-        <v>21.34</v>
+        <v>17.42</v>
       </c>
       <c r="K115" t="str">
         <v>AM sample (7-9am).</v>
@@ -3812,10 +3815,10 @@
         <v>510</v>
       </c>
       <c r="G116">
-        <v>99</v>
+        <v>170</v>
       </c>
       <c r="H116">
-        <v>561</v>
+        <v>450</v>
       </c>
       <c r="K116" t="str">
         <v>Declines ~2%/yr after age 25.</v>
@@ -3841,10 +3844,10 @@
         <v>320</v>
       </c>
       <c r="G117">
-        <v>40.5</v>
+        <v>86.25</v>
       </c>
       <c r="H117">
-        <v>352</v>
+        <v>278.75</v>
       </c>
       <c r="K117" t="str">
         <v>Declines ~2%/yr after age 25.</v>
@@ -3870,10 +3873,10 @@
         <v>360</v>
       </c>
       <c r="G118">
-        <v>81</v>
+        <v>130.5</v>
       </c>
       <c r="H118">
-        <v>396</v>
+        <v>319.5</v>
       </c>
       <c r="K118" t="str">
         <v>Age-adjusted: 16-24 ~182-780; 25-39 ~114-492; 40-54 ~90-360; 55+ ~71-290.</v>
@@ -3899,7 +3902,7 @@
         <v>15</v>
       </c>
       <c r="H119">
-        <v>20</v>
+        <v>12.75</v>
       </c>
       <c r="K119" t="str">
         <v>Optimal &lt;10.</v>
@@ -3925,7 +3928,7 @@
         <v>0.5</v>
       </c>
       <c r="H120">
-        <v>0.55</v>
+        <v>0.425</v>
       </c>
       <c r="K120" t="str">
         <v>Oxidative stress; higher = more damage. Highly method/assay-dependent.</v>
@@ -3951,7 +3954,7 @@
         <v>1</v>
       </c>
       <c r="H121">
-        <v>3</v>
+        <v>0.85</v>
       </c>
       <c r="K121" t="str">
         <v>Cardiac risk: &lt;1 low, 1-3 average, &gt;3 high.</v>
@@ -3977,10 +3980,10 @@
         <v>24.9</v>
       </c>
       <c r="G122">
-        <v>2.34</v>
+        <v>5.945</v>
       </c>
       <c r="H122">
-        <v>27.39</v>
+        <v>21.555</v>
       </c>
       <c r="K122" t="str">
         <v>Optimal &lt;10; insulin-resistant pattern &gt;15.</v>
@@ -4006,7 +4009,7 @@
         <v>5</v>
       </c>
       <c r="H123">
-        <v>5.5</v>
+        <v>4.25</v>
       </c>
       <c r="K123" t="str">
         <v>Pulsatile; random/fasting typically low.</v>
@@ -4032,9 +4035,12 @@
         <v>100</v>
       </c>
       <c r="G124">
-        <v>20</v>
+        <v>40.5</v>
       </c>
       <c r="H124">
+        <v>89.5</v>
+      </c>
+      <c r="J124">
         <v>150</v>
       </c>
       <c r="K124" t="str">
@@ -4061,10 +4067,10 @@
         <v>65</v>
       </c>
       <c r="G125">
-        <v>13.5</v>
+        <v>22.5</v>
       </c>
       <c r="H125">
-        <v>71.5</v>
+        <v>57.5</v>
       </c>
       <c r="K125" t="str">
         <v>Interpret with calcium, phosphorus, vitamin D.</v>
@@ -4090,7 +4096,7 @@
         <v>7</v>
       </c>
       <c r="H126">
-        <v>7.7</v>
+        <v>5.95</v>
       </c>
       <c r="K126" t="str">
         <v>High-sensitivity assays ULN ~1.8.</v>
@@ -4116,7 +4122,7 @@
         <v>8.1</v>
       </c>
       <c r="H127">
-        <v>8.91</v>
+        <v>6.885</v>
       </c>
       <c r="K127" t="str">
         <v/>
@@ -4142,10 +4148,10 @@
         <v>400</v>
       </c>
       <c r="G128">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="H128">
-        <v>440</v>
+        <v>370</v>
       </c>
       <c r="K128" t="str">
         <v/>
@@ -4171,7 +4177,7 @@
         <v>15</v>
       </c>
       <c r="H129">
-        <v>16.5</v>
+        <v>12.75</v>
       </c>
       <c r="K129" t="str">
         <v/>
@@ -4197,7 +4203,7 @@
         <v>20</v>
       </c>
       <c r="H130">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K130" t="str">
         <v/>
@@ -4258,7 +4264,7 @@
         <v>14</v>
       </c>
       <c r="H132">
-        <v>15.4</v>
+        <v>11.9</v>
       </c>
       <c r="K132" t="str">
         <v/>
@@ -4284,10 +4290,10 @@
         <v>180</v>
       </c>
       <c r="G133">
-        <v>81</v>
+        <v>103.5</v>
       </c>
       <c r="H133">
-        <v>198</v>
+        <v>166.5</v>
       </c>
       <c r="K133" t="str">
         <v/>
@@ -4313,10 +4319,10 @@
         <v>45</v>
       </c>
       <c r="G134">
-        <v>12.6</v>
+        <v>18.65</v>
       </c>
       <c r="H134">
-        <v>49.5</v>
+        <v>40.35</v>
       </c>
       <c r="K134" t="str">
         <v/>
@@ -4342,10 +4348,10 @@
         <v>4.8</v>
       </c>
       <c r="G135">
-        <v>0.9</v>
+        <v>1.57</v>
       </c>
       <c r="H135">
-        <v>5.28</v>
+        <v>4.23</v>
       </c>
       <c r="K135" t="str">
         <v>Absolute lymphocyte count.</v>
@@ -4371,7 +4377,7 @@
         <v>500</v>
       </c>
       <c r="H136">
-        <v>550</v>
+        <v>425</v>
       </c>
       <c r="K136" t="str">
         <v>FEU; &gt;500 suggests active clotting.</v>
@@ -4397,7 +4403,7 @@
         <v>15</v>
       </c>
       <c r="H137">
-        <v>20</v>
+        <v>12.75</v>
       </c>
       <c r="K137" t="str">
         <v>Optimal &lt;10.</v>
@@ -4423,10 +4429,10 @@
         <v>171</v>
       </c>
       <c r="G138">
-        <v>31.5</v>
+        <v>55.4</v>
       </c>
       <c r="H138">
-        <v>188.1</v>
+        <v>150.6</v>
       </c>
       <c r="K138" t="str">
         <v>Deficiency &lt;40; investigate &lt;70.</v>
@@ -4452,10 +4458,10 @@
         <v>903</v>
       </c>
       <c r="G139">
-        <v>252</v>
+        <v>373.45</v>
       </c>
       <c r="H139">
-        <v>993.3</v>
+        <v>809.55</v>
       </c>
       <c r="K139" t="str">
         <v/>
@@ -4481,10 +4487,10 @@
         <v>4.5</v>
       </c>
       <c r="G140">
-        <v>0.1</v>
+        <v>1.057</v>
       </c>
       <c r="H140">
-        <v>10</v>
+        <v>3.893</v>
       </c>
       <c r="I140">
         <v>0.01</v>
@@ -4516,10 +4522,10 @@
         <v>4.4</v>
       </c>
       <c r="G141">
-        <v>1.8</v>
+        <v>2.36</v>
       </c>
       <c r="H141">
-        <v>4.84</v>
+        <v>4.04</v>
       </c>
       <c r="K141" t="str">
         <v/>
@@ -4545,10 +4551,10 @@
         <v>1.77</v>
       </c>
       <c r="G142">
-        <v>0.738</v>
+        <v>0.962</v>
       </c>
       <c r="H142">
-        <v>1.947</v>
+        <v>1.628</v>
       </c>
       <c r="K142" t="str">
         <v/>
@@ -4574,10 +4580,10 @@
         <v>19.4</v>
       </c>
       <c r="G143">
-        <v>5.58</v>
+        <v>8.18</v>
       </c>
       <c r="H143">
-        <v>21.34</v>
+        <v>17.42</v>
       </c>
       <c r="K143" t="str">
         <v>AM sample (7-9am).</v>
@@ -4603,10 +4609,10 @@
         <v>11.9</v>
       </c>
       <c r="G144">
-        <v>2.07</v>
+        <v>3.74</v>
       </c>
       <c r="H144">
-        <v>13.09</v>
+        <v>10.46</v>
       </c>
       <c r="K144" t="str">
         <v>PM sample; ~half of AM.</v>
@@ -4632,10 +4638,10 @@
         <v>99</v>
       </c>
       <c r="G145">
-        <v>60</v>
+        <v>74.35</v>
       </c>
       <c r="H145">
-        <v>125</v>
+        <v>94.65</v>
       </c>
       <c r="I145">
         <v>50</v>
@@ -4667,10 +4673,10 @@
         <v>24.9</v>
       </c>
       <c r="G146">
-        <v>2.34</v>
+        <v>5.945</v>
       </c>
       <c r="H146">
-        <v>27.39</v>
+        <v>21.555</v>
       </c>
       <c r="K146" t="str">
         <v>Optimal &lt;10; insulin-resistant pattern &gt;15.</v>
@@ -4696,9 +4702,12 @@
         <v>100</v>
       </c>
       <c r="G147">
-        <v>20</v>
+        <v>40.5</v>
       </c>
       <c r="H147">
+        <v>89.5</v>
+      </c>
+      <c r="J147">
         <v>150</v>
       </c>
       <c r="K147" t="str">
@@ -4760,7 +4769,7 @@
         <v>1</v>
       </c>
       <c r="H149">
-        <v>3</v>
+        <v>0.85</v>
       </c>
       <c r="K149" t="str">
         <v>Cardiac risk: &lt;1 low, 1-3 average, &gt;3 high.</v>
@@ -4786,10 +4795,10 @@
         <v>61</v>
       </c>
       <c r="G150">
-        <v>7.2</v>
+        <v>15.95</v>
       </c>
       <c r="H150">
-        <v>67.1</v>
+        <v>53.05</v>
       </c>
       <c r="K150" t="str">
         <v>Female upper ~36.</v>
@@ -4815,10 +4824,10 @@
         <v>280</v>
       </c>
       <c r="G151">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="H151">
-        <v>308</v>
+        <v>259</v>
       </c>
       <c r="K151" t="str">
         <v/>
@@ -4844,10 +4853,10 @@
         <v>110</v>
       </c>
       <c r="G152">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H152">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="K152" t="str">
         <v/>
@@ -4873,10 +4882,10 @@
         <v>140</v>
       </c>
       <c r="G153">
-        <v>9</v>
+        <v>29.5</v>
       </c>
       <c r="H153">
-        <v>154</v>
+        <v>120.5</v>
       </c>
       <c r="K153" t="str">
         <v/>
@@ -4937,7 +4946,7 @@
         <v>20</v>
       </c>
       <c r="H155">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K155" t="str">
         <v>&lt;20 negative (assay-dependent).</v>
@@ -4963,7 +4972,7 @@
         <v>4</v>
       </c>
       <c r="H156">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="K156" t="str">
         <v>&lt;4 negative; 4-10 weak positive; &gt;10 positive.</v>
@@ -4989,7 +4998,7 @@
         <v>50</v>
       </c>
       <c r="H157">
-        <v>55</v>
+        <v>42.5</v>
       </c>
       <c r="K157" t="str">
         <v>50-120 borderline; &gt;120 active GI inflammation (web research).</v>
@@ -5015,10 +5024,10 @@
         <v>1.1</v>
       </c>
       <c r="G158">
-        <v>0.72</v>
+        <v>0.845</v>
       </c>
       <c r="H158">
-        <v>1.21</v>
+        <v>1.055</v>
       </c>
       <c r="J158">
         <v>5</v>
@@ -5047,7 +5056,7 @@
         <v>0.3</v>
       </c>
       <c r="H159">
-        <v>0.33</v>
+        <v>0.255</v>
       </c>
       <c r="K159" t="str">
         <v/>
@@ -5073,10 +5082,10 @@
         <v>0.9</v>
       </c>
       <c r="G160">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
       <c r="H160">
-        <v>0.99</v>
+        <v>0.78</v>
       </c>
       <c r="K160" t="str">
         <v/>

</xml_diff>